<commit_message>
Fixed NBA Standings Tiebreakers
</commit_message>
<xml_diff>
--- a/DBs/wnba/Results/WNBA_2010_Results.xlsx
+++ b/DBs/wnba/Results/WNBA_2010_Results.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tjsut\TracerSports\WNBA_Elo\Results\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tjsut\tracersports-app\DBs\wnba\Results\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7E4634EB-2F3C-463E-9949-3F7FEE5027F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F08E50CF-FC28-4768-B4A7-94BD5D7E5B6A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{1654EDFA-4626-4D72-A032-E72CC9A130FE}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2210" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2178" uniqueCount="27">
   <si>
     <t>Date</t>
   </si>
@@ -117,6 +117,9 @@
   </si>
   <si>
     <t>TUL</t>
+  </si>
+  <si>
+    <t>P</t>
   </si>
 </sst>
 </file>
@@ -13621,10 +13624,10 @@
         <v>2010</v>
       </c>
       <c r="C410" t="s">
-        <v>10</v>
-      </c>
-      <c r="D410" t="s">
-        <v>11</v>
+        <v>26</v>
+      </c>
+      <c r="D410">
+        <v>1</v>
       </c>
       <c r="E410" t="s">
         <v>17</v>
@@ -13653,10 +13656,10 @@
         <v>2010</v>
       </c>
       <c r="C411" t="s">
-        <v>10</v>
-      </c>
-      <c r="D411" t="s">
-        <v>11</v>
+        <v>26</v>
+      </c>
+      <c r="D411">
+        <v>1</v>
       </c>
       <c r="E411" t="s">
         <v>19</v>
@@ -13685,10 +13688,10 @@
         <v>2010</v>
       </c>
       <c r="C412" t="s">
-        <v>10</v>
-      </c>
-      <c r="D412" t="s">
-        <v>11</v>
+        <v>26</v>
+      </c>
+      <c r="D412">
+        <v>1</v>
       </c>
       <c r="E412" t="s">
         <v>24</v>
@@ -13717,10 +13720,10 @@
         <v>2010</v>
       </c>
       <c r="C413" t="s">
-        <v>10</v>
-      </c>
-      <c r="D413" t="s">
-        <v>11</v>
+        <v>26</v>
+      </c>
+      <c r="D413">
+        <v>1</v>
       </c>
       <c r="E413" t="s">
         <v>12</v>
@@ -13749,10 +13752,10 @@
         <v>2010</v>
       </c>
       <c r="C414" t="s">
-        <v>10</v>
-      </c>
-      <c r="D414" t="s">
-        <v>11</v>
+        <v>26</v>
+      </c>
+      <c r="D414">
+        <v>1</v>
       </c>
       <c r="E414" t="s">
         <v>20</v>
@@ -13781,10 +13784,10 @@
         <v>2010</v>
       </c>
       <c r="C415" t="s">
-        <v>10</v>
-      </c>
-      <c r="D415" t="s">
-        <v>11</v>
+        <v>26</v>
+      </c>
+      <c r="D415">
+        <v>1</v>
       </c>
       <c r="E415" t="s">
         <v>15</v>
@@ -13813,10 +13816,10 @@
         <v>2010</v>
       </c>
       <c r="C416" t="s">
-        <v>10</v>
-      </c>
-      <c r="D416" t="s">
-        <v>11</v>
+        <v>26</v>
+      </c>
+      <c r="D416">
+        <v>1</v>
       </c>
       <c r="E416" t="s">
         <v>22</v>
@@ -13845,10 +13848,10 @@
         <v>2010</v>
       </c>
       <c r="C417" t="s">
-        <v>10</v>
-      </c>
-      <c r="D417" t="s">
-        <v>11</v>
+        <v>26</v>
+      </c>
+      <c r="D417">
+        <v>1</v>
       </c>
       <c r="E417" t="s">
         <v>16</v>
@@ -13877,10 +13880,10 @@
         <v>2010</v>
       </c>
       <c r="C418" t="s">
-        <v>10</v>
-      </c>
-      <c r="D418" t="s">
-        <v>11</v>
+        <v>26</v>
+      </c>
+      <c r="D418">
+        <v>1</v>
       </c>
       <c r="E418" t="s">
         <v>12</v>
@@ -13909,10 +13912,10 @@
         <v>2010</v>
       </c>
       <c r="C419" t="s">
-        <v>10</v>
-      </c>
-      <c r="D419" t="s">
-        <v>11</v>
+        <v>26</v>
+      </c>
+      <c r="D419">
+        <v>1</v>
       </c>
       <c r="E419" t="s">
         <v>24</v>
@@ -13941,10 +13944,10 @@
         <v>2010</v>
       </c>
       <c r="C420" t="s">
-        <v>10</v>
-      </c>
-      <c r="D420" t="s">
-        <v>11</v>
+        <v>26</v>
+      </c>
+      <c r="D420">
+        <v>1</v>
       </c>
       <c r="E420" t="s">
         <v>19</v>
@@ -13973,10 +13976,10 @@
         <v>2010</v>
       </c>
       <c r="C421" t="s">
-        <v>10</v>
-      </c>
-      <c r="D421" t="s">
-        <v>11</v>
+        <v>26</v>
+      </c>
+      <c r="D421">
+        <v>1</v>
       </c>
       <c r="E421" t="s">
         <v>17</v>
@@ -14005,10 +14008,10 @@
         <v>2010</v>
       </c>
       <c r="C422" t="s">
-        <v>10</v>
-      </c>
-      <c r="D422" t="s">
-        <v>11</v>
+        <v>26</v>
+      </c>
+      <c r="D422">
+        <v>1</v>
       </c>
       <c r="E422" t="s">
         <v>16</v>
@@ -14037,10 +14040,10 @@
         <v>2010</v>
       </c>
       <c r="C423" t="s">
-        <v>10</v>
-      </c>
-      <c r="D423" t="s">
-        <v>11</v>
+        <v>26</v>
+      </c>
+      <c r="D423">
+        <v>1</v>
       </c>
       <c r="E423" t="s">
         <v>22</v>
@@ -14069,10 +14072,10 @@
         <v>2010</v>
       </c>
       <c r="C424" t="s">
-        <v>10</v>
-      </c>
-      <c r="D424" t="s">
-        <v>11</v>
+        <v>26</v>
+      </c>
+      <c r="D424">
+        <v>1</v>
       </c>
       <c r="E424" t="s">
         <v>15</v>
@@ -14101,10 +14104,10 @@
         <v>2010</v>
       </c>
       <c r="C425" t="s">
-        <v>10</v>
-      </c>
-      <c r="D425" t="s">
-        <v>11</v>
+        <v>26</v>
+      </c>
+      <c r="D425">
+        <v>1</v>
       </c>
       <c r="E425" t="s">
         <v>20</v>
@@ -14133,10 +14136,10 @@
         <v>2010</v>
       </c>
       <c r="C426" t="s">
-        <v>10</v>
-      </c>
-      <c r="D426" t="s">
-        <v>11</v>
+        <v>26</v>
+      </c>
+      <c r="D426">
+        <v>1</v>
       </c>
       <c r="E426" t="s">
         <v>20</v>
@@ -14165,10 +14168,10 @@
         <v>2010</v>
       </c>
       <c r="C427" t="s">
-        <v>10</v>
-      </c>
-      <c r="D427" t="s">
-        <v>11</v>
+        <v>26</v>
+      </c>
+      <c r="D427">
+        <v>1</v>
       </c>
       <c r="E427" t="s">
         <v>15</v>
@@ -14197,10 +14200,10 @@
         <v>2010</v>
       </c>
       <c r="C428" t="s">
-        <v>10</v>
-      </c>
-      <c r="D428" t="s">
-        <v>11</v>
+        <v>26</v>
+      </c>
+      <c r="D428">
+        <v>2</v>
       </c>
       <c r="E428" t="s">
         <v>16</v>
@@ -14229,10 +14232,10 @@
         <v>2010</v>
       </c>
       <c r="C429" t="s">
-        <v>10</v>
-      </c>
-      <c r="D429" t="s">
-        <v>11</v>
+        <v>26</v>
+      </c>
+      <c r="D429">
+        <v>2</v>
       </c>
       <c r="E429" t="s">
         <v>19</v>
@@ -14261,10 +14264,10 @@
         <v>2010</v>
       </c>
       <c r="C430" t="s">
-        <v>10</v>
-      </c>
-      <c r="D430" t="s">
-        <v>11</v>
+        <v>26</v>
+      </c>
+      <c r="D430">
+        <v>2</v>
       </c>
       <c r="E430" t="s">
         <v>24</v>
@@ -14293,10 +14296,10 @@
         <v>2010</v>
       </c>
       <c r="C431" t="s">
-        <v>10</v>
-      </c>
-      <c r="D431" t="s">
-        <v>11</v>
+        <v>26</v>
+      </c>
+      <c r="D431">
+        <v>2</v>
       </c>
       <c r="E431" t="s">
         <v>15</v>
@@ -14325,10 +14328,10 @@
         <v>2010</v>
       </c>
       <c r="C432" t="s">
-        <v>10</v>
-      </c>
-      <c r="D432" t="s">
-        <v>11</v>
+        <v>26</v>
+      </c>
+      <c r="D432">
+        <v>2</v>
       </c>
       <c r="E432" t="s">
         <v>19</v>
@@ -14357,10 +14360,10 @@
         <v>2010</v>
       </c>
       <c r="C433" t="s">
-        <v>10</v>
-      </c>
-      <c r="D433" t="s">
-        <v>11</v>
+        <v>26</v>
+      </c>
+      <c r="D433">
+        <v>2</v>
       </c>
       <c r="E433" t="s">
         <v>16</v>
@@ -14389,10 +14392,10 @@
         <v>2010</v>
       </c>
       <c r="C434" t="s">
-        <v>10</v>
-      </c>
-      <c r="D434" t="s">
-        <v>11</v>
+        <v>26</v>
+      </c>
+      <c r="D434">
+        <v>2</v>
       </c>
       <c r="E434" t="s">
         <v>15</v>
@@ -14421,10 +14424,10 @@
         <v>2010</v>
       </c>
       <c r="C435" t="s">
-        <v>10</v>
-      </c>
-      <c r="D435" t="s">
-        <v>11</v>
+        <v>26</v>
+      </c>
+      <c r="D435">
+        <v>2</v>
       </c>
       <c r="E435" t="s">
         <v>24</v>
@@ -14453,10 +14456,10 @@
         <v>2010</v>
       </c>
       <c r="C436" t="s">
-        <v>10</v>
-      </c>
-      <c r="D436" t="s">
-        <v>11</v>
+        <v>26</v>
+      </c>
+      <c r="D436">
+        <v>3</v>
       </c>
       <c r="E436" t="s">
         <v>24</v>
@@ -14485,10 +14488,10 @@
         <v>2010</v>
       </c>
       <c r="C437" t="s">
-        <v>10</v>
-      </c>
-      <c r="D437" t="s">
-        <v>11</v>
+        <v>26</v>
+      </c>
+      <c r="D437">
+        <v>3</v>
       </c>
       <c r="E437" t="s">
         <v>19</v>
@@ -14517,10 +14520,10 @@
         <v>2010</v>
       </c>
       <c r="C438" t="s">
-        <v>10</v>
-      </c>
-      <c r="D438" t="s">
-        <v>11</v>
+        <v>26</v>
+      </c>
+      <c r="D438">
+        <v>3</v>
       </c>
       <c r="E438" t="s">
         <v>24</v>
@@ -14549,10 +14552,10 @@
         <v>2010</v>
       </c>
       <c r="C439" t="s">
-        <v>10</v>
-      </c>
-      <c r="D439" t="s">
-        <v>11</v>
+        <v>26</v>
+      </c>
+      <c r="D439">
+        <v>3</v>
       </c>
       <c r="E439" t="s">
         <v>19</v>
@@ -14581,10 +14584,10 @@
         <v>2010</v>
       </c>
       <c r="C440" t="s">
-        <v>10</v>
-      </c>
-      <c r="D440" t="s">
-        <v>11</v>
+        <v>26</v>
+      </c>
+      <c r="D440">
+        <v>3</v>
       </c>
       <c r="E440" t="s">
         <v>19</v>
@@ -14613,10 +14616,10 @@
         <v>2010</v>
       </c>
       <c r="C441" t="s">
-        <v>10</v>
-      </c>
-      <c r="D441" t="s">
-        <v>11</v>
+        <v>26</v>
+      </c>
+      <c r="D441">
+        <v>3</v>
       </c>
       <c r="E441" t="s">
         <v>24</v>

</xml_diff>